<commit_message>
corrección en plantilla 7000 recaudado
</commit_message>
<xml_diff>
--- a/public/Guia/7000-Recaudado-CuentasConceptos.xlsx
+++ b/public/Guia/7000-Recaudado-CuentasConceptos.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Dmijangos\Documents\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5A85BE93-948F-4CA5-8558-8DA4BDECB435}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A80DCC5-FB95-440E-8A40-C6171C96BFAE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="20">
   <si>
     <t>cuenta</t>
   </si>
@@ -57,15 +57,6 @@
   </si>
   <si>
     <t>Contable - Abono</t>
-  </si>
-  <si>
-    <t>5.2.5.9.01.04</t>
-  </si>
-  <si>
-    <t>III.1.4 TRANSFERENCIAS, ASIGNACIONES, SUBSIDIOS Y OTRAS AYUDAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Por el devengado por prestaciones de pensiones y jubilaciones </t>
   </si>
   <si>
     <t>Contable - Cargo</t>
@@ -513,97 +504,97 @@
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D2" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="B3" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D3" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="B4" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D4" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" t="s">
+        <v>19</v>
+      </c>
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B5" t="s">
-        <v>22</v>
-      </c>
-      <c r="C5" s="2" t="s">
-        <v>17</v>
-      </c>
       <c r="D5" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="4" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D6" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D7" t="s">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D8" t="s">
         <v>6</v>
@@ -611,13 +602,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D9" t="s">
         <v>6</v>
@@ -625,13 +616,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B10" t="s">
         <v>19</v>
       </c>
-      <c r="B10" t="s">
-        <v>22</v>
-      </c>
       <c r="C10" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D10" t="s">
         <v>5</v>
@@ -639,13 +630,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="B11" t="s">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="D11" t="s">
         <v>4</v>
@@ -956,15 +947,9 @@
       <c r="C72" s="2"/>
     </row>
     <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B73" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="C73" s="2" t="s">
-        <v>9</v>
-      </c>
+      <c r="A73" s="1"/>
+      <c r="B73" s="2"/>
+      <c r="C73" s="2"/>
     </row>
     <row r="74" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A74" s="1"/>

</xml_diff>